<commit_message>
Integrazione scadenziario e interventi
</commit_message>
<xml_diff>
--- a/FileRaw/scadenziario.xlsx
+++ b/FileRaw/scadenziario.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utente\OneDrive - CCH SRL (1)\Attachments\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreadepaoli/Documents/Coding/cDen/chipdent/FileRaw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E1A339F-0977-460D-A068-32E0DF034CFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2AEBC7F-2B6C-3643-80CA-86D92C4E99BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8CD124A1-1CB5-4FF2-979A-EA8B3073B6D3}"/>
+    <workbookView xWindow="160" yWindow="720" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8CD124A1-1CB5-4FF2-979A-EA8B3073B6D3}"/>
   </bookViews>
   <sheets>
     <sheet name="prova" sheetId="2" r:id="rId1"/>
+    <sheet name="chiarimenti sul file" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">prova!$A$1:$O$1</definedName>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="964" uniqueCount="376">
   <si>
     <t>DATA</t>
   </si>
@@ -926,6 +927,965 @@
   </si>
   <si>
     <t>AQ03811636</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>Colonna</t>
+  </si>
+  <si>
+    <t>Domanda</t>
+  </si>
+  <si>
+    <t>Note / Ipotesi mia</t>
+  </si>
+  <si>
+    <t>Feedback Confident</t>
+  </si>
+  <si>
+    <r>
+      <t>È sempre la </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>data di scadenza</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> del pagamento? Può essere data fattura o data pagamento?</t>
+    </r>
+  </si>
+  <si>
+    <t>Tutte le righe sono "Pagato": ci serve sapere se è la scadenza o il pagato effettivo</t>
+  </si>
+  <si>
+    <r>
+      <t>Per le righe già pagate, conservate da qualche parte la </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>data di pagamento effettivo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>?</t>
+    </r>
+  </si>
+  <si>
+    <t>Se no, la consideriamo coincidente con questa colonna</t>
+  </si>
+  <si>
+    <r>
+      <t>Possiamo avere l'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>elenco completo delle sigle</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> e a quale sede corrispondono?</t>
+    </r>
+  </si>
+  <si>
+    <t>Trovate: BOL, BUS, CCH, COM, COR, DES, GIU, MI3, MI6, MI7, MI9, SGM, VAR</t>
+  </si>
+  <si>
+    <r>
+      <t>BOL</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>=Bologna? </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>GIU</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>=? </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>SGM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>=? </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>COR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>=?</t>
+    </r>
+  </si>
+  <si>
+    <t>Da confermare una a una</t>
+  </si>
+  <si>
+    <r>
+      <t>CCH</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> è una sede o è la </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>holding/società</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>? Vedo anche "CCH SRL" come fornitore</t>
+    </r>
+  </si>
+  <si>
+    <t>Probabilmente è la holding</t>
+  </si>
+  <si>
+    <t>Per costi di gruppo/cross-sede esiste una sigla "tutte le sedi"?</t>
+  </si>
+  <si>
+    <t>Oggi non c'è</t>
+  </si>
+  <si>
+    <r>
+      <t>Cosa significano i 4 valori </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>E</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>M</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>O</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>?</t>
+    </r>
+  </si>
+  <si>
+    <t>L'header dice "E/M" ma trovo anche A e O</t>
+  </si>
+  <si>
+    <r>
+      <t>Ipotesi nostra: E=Emessa, M=Manuale. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> e </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>O</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>?</t>
+    </r>
+  </si>
+  <si>
+    <t>Da confermare</t>
+  </si>
+  <si>
+    <r>
+      <t>Significa </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>Bonifico Manuale</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>? Solo quando il bonifico va eseguito a mano?</t>
+    </r>
+  </si>
+  <si>
+    <t>Solo valore "BM" o vuoto</t>
+  </si>
+  <si>
+    <r>
+      <t>Se BM è "manuale", </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>lo escludiamo dalla distinta SEPA automatica</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>?</t>
+    </r>
+  </si>
+  <si>
+    <t>Confermare logica</t>
+  </si>
+  <si>
+    <t>(n° doc)</t>
+  </si>
+  <si>
+    <r>
+      <t>La colonna senza header è il </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>numero documento</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>?</t>
+    </r>
+  </si>
+  <si>
+    <t>Sì, immaginiamo</t>
+  </si>
+  <si>
+    <r>
+      <t>Va bene importare come </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>testo libero</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> o serve un campo strutturato separato?</t>
+    </r>
+  </si>
+  <si>
+    <t>Trovo numeri, codici lunghi, testi tipo "Compenso Amministratore"</t>
+  </si>
+  <si>
+    <r>
+      <t>Alcune celle hanno </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>tab e a-capo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> dentro: li ripuliamo o sono significativi?</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Es. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>\t\n0100220240017351500</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>È l'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>imponibile</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> (al netto IVA), giusto?</t>
+    </r>
+  </si>
+  <si>
+    <t>Sì, ipotizzo</t>
+  </si>
+  <si>
+    <r>
+      <t>È l'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>importo IVA in euro</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> (non l'aliquota)?</t>
+    </r>
+  </si>
+  <si>
+    <t>Es. 14,96 € — sembra in euro</t>
+  </si>
+  <si>
+    <r>
+      <t>Quando è </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> o vuota → operazione esente (compensi, F24, ritenute)? Va bene importarla come IVA = 0?</t>
+    </r>
+  </si>
+  <si>
+    <t>Confermare</t>
+  </si>
+  <si>
+    <r>
+      <t>È sempre </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>IMPORTO + IVA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>?</t>
+    </r>
+  </si>
+  <si>
+    <t>Da confermare per evitare disallineamenti</t>
+  </si>
+  <si>
+    <r>
+      <t>Oltre a Bonifico/RID/RIBA/CC/Contanti/F24 ne usate </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>altri</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> (Assegno, Compensazione, PayPal, …)?</t>
+    </r>
+  </si>
+  <si>
+    <t>Lista da chiudere</t>
+  </si>
+  <si>
+    <r>
+      <t>CC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> significa </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>Carta di Credito</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> o </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>Conto Corrente</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>?</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Quali sono </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>tutti i possibili valori</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> (Da Pagare, Programmato, Scaduto, Annullato, …) e come li scrivete?</t>
+    </r>
+  </si>
+  <si>
+    <t>Nel file solo "Pagato"</t>
+  </si>
+  <si>
+    <r>
+      <t>Le 33 categorie sono una </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>lista chiusa</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> o ne aggiungete spesso?</t>
+    </r>
+  </si>
+  <si>
+    <t>Per decidere se enum o tabella</t>
+  </si>
+  <si>
+    <r>
+      <t>Voci che sembrano ricavi (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>ALTRI RICAVI VARI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>DIVIDENDI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>ENTRANCE FEE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>FONDO INVESTIMENTO</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>) cosa rappresentano nello scadenziario passivo?</t>
+    </r>
+  </si>
+  <si>
+    <t>Errore di registrazione o logica precisa?</t>
+  </si>
+  <si>
+    <r>
+      <t>MEDICI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>DIREZIONE SANITARIA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>COMPENSO AMMINISTRATORE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>COMPENSO CONSIGLIERE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> → li gestiamo come </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>dottori-fornitori</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> o fornitore generico?</t>
+    </r>
+  </si>
+  <si>
+    <t>Sono persone fisiche/soci</t>
+  </si>
+  <si>
+    <r>
+      <t>Le </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>ritenute</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> (es. "RITENUTE NUNZIATI" con F24) sono righe indipendenti o "figlie" del compenso a cui si riferiscono?</t>
+    </r>
+  </si>
+  <si>
+    <t>Da decidere il modello</t>
+  </si>
+  <si>
+    <t>NOTE</t>
+  </si>
+  <si>
+    <t>Importazione 1:1 come testo libero, ok?</t>
+  </si>
+  <si>
+    <r>
+      <t>Quando è vuoto è </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>normale</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> (CC/F24/Contanti) o è "da recuperare"?</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>È sempre l'IBAN del </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>fornitore</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t> (da anagrafica) o può variare scadenza per scadenza?</t>
+    </r>
+  </si>
+  <si>
+    <t>Decide se snapshot o ref</t>
+  </si>
+  <si>
+    <t>Data Pagamento previsto</t>
+  </si>
+  <si>
+    <t>No e a volte può differire ma non mi serve sapere la data del pagamento effettivo</t>
+  </si>
+  <si>
+    <t>BOL, BUS, CCH, COM, COR, DES, GIU, MI3, MI6, MI7, MI9, SGM, VAR, BRU, CMS, CAS - le sigle si aggiungono quando una clinica viene aperta</t>
+  </si>
+  <si>
+    <t>DES ( Desio): IDENT SRL
+VAR: (Varese): IDENT VARESE SRL
+GIU: (Giussano): IDENT GIUSSANO SRL
+COR: (Cormano): IDENT CORMANO SRL
+COM: (Como): IDENT COMO SRL
+MI7:  IDENT MILANO7 SRL
+MI9: IDENT MILANO9 SRL
+SGM: (San Giuliano): IDENT SGM SRL
+BUS: (Busto Arsizio): IDENT BUSTO ARSIZIO SRL
+BOL: (Bollate): IDENT BOLLATE SRL
+MI6: IDENT MILANO6 SRL
+Mi3: IDENT MILANO3 SRL
+BRU: (Brugherio): IDENT BRUGHERIO SRL
+CMS: (Comasina): IDENT COMASINA SRL</t>
+  </si>
+  <si>
+    <t>CCH è la holding ma comunque una società che fa pagamenti.</t>
+  </si>
+  <si>
+    <t>No, sono divise per studi/CCH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E: elettronico - M: manuale </t>
+  </si>
+  <si>
+    <t>BM - bonifco multiplo CBI</t>
+  </si>
+  <si>
+    <t>Vedi sopra</t>
+  </si>
+  <si>
+    <t>Numero fattura o causale bonifico</t>
+  </si>
+  <si>
+    <t>Tutto significativo</t>
+  </si>
+  <si>
+    <t>IVA è un costo per tutte le sedi - per CCH tracciamo invece l'IVA</t>
+  </si>
+  <si>
+    <t>si viene riportato l'importo dell'IVA</t>
+  </si>
+  <si>
+    <t>Quando IVA è vuota vuol dire che l'IVA è già inserita perchè un costo</t>
+  </si>
+  <si>
+    <t>come da scad</t>
+  </si>
+  <si>
+    <t>carta di credito</t>
+  </si>
+  <si>
+    <t>Da pagare, Pagato, Mai pagato</t>
+  </si>
+  <si>
+    <t>Chiusa</t>
+  </si>
+  <si>
+    <t>Logica precisa</t>
+  </si>
+  <si>
+    <t>No - tutti separati</t>
+  </si>
+  <si>
+    <t>Tutti gli F24 sono figli di un compenso o di una fattura</t>
+  </si>
+  <si>
+    <t>Non capisco la domanda</t>
+  </si>
+  <si>
+    <t>Se non è un bonifico non serve IBAN</t>
+  </si>
+  <si>
+    <t>Normalmente è sempre uguale</t>
   </si>
 </sst>
 </file>
@@ -937,7 +1897,7 @@
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-410]_-;\-* #,##0.00\ [$€-410]_-;_-* &quot;-&quot;??\ [$€-410]_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="&quot; € &quot;#,##0.00\ ;&quot;-€ &quot;#,##0.00\ ;&quot; € -&quot;#\ ;@\ "/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -981,21 +1941,96 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Courier New"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -1005,7 +2040,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyProtection="1">
       <protection locked="0"/>
@@ -1180,12 +2215,43 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
+    <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Euro" xfId="3" xr:uid="{5471AE4C-B81C-4277-AFBB-4B7D11EDD6D9}"/>
     <cellStyle name="Excel Built-in Normal" xfId="2" xr:uid="{CA55FD1A-2FB4-46CF-A791-D2690E0F8B92}"/>
-    <cellStyle name="Normale" xfId="0" builtinId="0"/>
-    <cellStyle name="Valuta" xfId="1" builtinId="4"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1201,7 +2267,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema di Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1518,27 +2584,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FD43689-4205-4B1F-A2C0-F6B0035B0816}">
   <dimension ref="A1:Q95"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="41.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="55.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.83203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="30.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="41.85546875" customWidth="1"/>
-    <col min="15" max="15" width="32.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="30.1640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="41.83203125" customWidth="1"/>
+    <col min="15" max="15" width="32.5" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="6" customFormat="1" ht="28.9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" s="6" customFormat="1" ht="29" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -1583,7 +2649,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="21">
         <v>45535</v>
       </c>
@@ -1630,7 +2696,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="21">
         <v>45667</v>
       </c>
@@ -1677,7 +2743,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="4" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="7">
         <v>45404</v>
       </c>
@@ -1716,7 +2782,7 @@
       </c>
       <c r="P4" s="5"/>
     </row>
-    <row r="5" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A5" s="7">
         <v>45411</v>
       </c>
@@ -1755,7 +2821,7 @@
       </c>
       <c r="P5" s="5"/>
     </row>
-    <row r="6" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A6" s="21">
         <v>45412</v>
       </c>
@@ -1798,7 +2864,7 @@
       </c>
       <c r="P6" s="5"/>
     </row>
-    <row r="7" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="21">
         <v>45412</v>
       </c>
@@ -1844,7 +2910,7 @@
       </c>
       <c r="P7" s="5"/>
     </row>
-    <row r="8" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A8" s="21">
         <v>45412</v>
       </c>
@@ -1888,7 +2954,7 @@
       <c r="O8" s="5"/>
       <c r="P8" s="5"/>
     </row>
-    <row r="9" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="21">
         <v>45412</v>
       </c>
@@ -1936,7 +3002,7 @@
       </c>
       <c r="P9" s="5"/>
     </row>
-    <row r="10" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A10" s="15">
         <v>45636</v>
       </c>
@@ -1980,7 +3046,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="15">
         <v>45636</v>
       </c>
@@ -2024,7 +3090,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A12" s="21">
         <v>45606</v>
       </c>
@@ -2072,7 +3138,7 @@
       </c>
       <c r="P12" s="5"/>
     </row>
-    <row r="13" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="21">
         <v>45626</v>
       </c>
@@ -2116,7 +3182,7 @@
       </c>
       <c r="P13" s="5"/>
     </row>
-    <row r="14" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="7">
         <v>45493</v>
       </c>
@@ -2158,7 +3224,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="7">
         <v>45493</v>
       </c>
@@ -2200,7 +3266,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A16" s="21">
         <v>45483</v>
       </c>
@@ -2246,7 +3312,7 @@
       </c>
       <c r="P16" s="5"/>
     </row>
-    <row r="17" spans="1:17" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:17" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A17" s="21">
         <v>45483</v>
       </c>
@@ -2292,7 +3358,7 @@
       </c>
       <c r="P17" s="5"/>
     </row>
-    <row r="18" spans="1:17" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:17" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="21">
         <v>45483</v>
       </c>
@@ -2338,7 +3404,7 @@
       </c>
       <c r="P18" s="5"/>
     </row>
-    <row r="19" spans="1:17" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:17" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A19" s="21">
         <v>45489</v>
       </c>
@@ -2376,7 +3442,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="20" spans="1:17" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:17" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A20" s="21">
         <v>45489</v>
       </c>
@@ -2414,7 +3480,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="21" spans="1:17" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:17" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A21" s="21">
         <v>45489</v>
       </c>
@@ -2452,7 +3518,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="22" spans="1:17" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:17" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A22" s="21">
         <v>45483</v>
       </c>
@@ -2496,7 +3562,7 @@
       </c>
       <c r="P22" s="5"/>
     </row>
-    <row r="23" spans="1:17" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:17" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="21">
         <v>45483</v>
       </c>
@@ -2541,7 +3607,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="24" spans="1:17" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:17" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A24" s="21">
         <v>45551</v>
       </c>
@@ -2578,7 +3644,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="25" spans="1:17" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:17" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="21">
         <v>45453</v>
       </c>
@@ -2623,7 +3689,7 @@
       <c r="P25" s="5"/>
       <c r="Q25" s="16"/>
     </row>
-    <row r="26" spans="1:17" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:17" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="21">
         <v>45453</v>
       </c>
@@ -2667,7 +3733,7 @@
       </c>
       <c r="P26" s="5"/>
     </row>
-    <row r="27" spans="1:17" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:17" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A27" s="21">
         <v>45453</v>
       </c>
@@ -2715,7 +3781,7 @@
       </c>
       <c r="P27" s="5"/>
     </row>
-    <row r="28" spans="1:17" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:17" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="21">
         <v>45443</v>
       </c>
@@ -2763,7 +3829,7 @@
       </c>
       <c r="P28" s="5"/>
     </row>
-    <row r="29" spans="1:17" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:17" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="21">
         <v>45443</v>
       </c>
@@ -2807,7 +3873,7 @@
       </c>
       <c r="P29" s="5"/>
     </row>
-    <row r="30" spans="1:17" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:17" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="21">
         <v>45443</v>
       </c>
@@ -2855,7 +3921,7 @@
       </c>
       <c r="P30" s="5"/>
     </row>
-    <row r="31" spans="1:17" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:17" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A31" s="7">
         <v>45443</v>
       </c>
@@ -2899,7 +3965,7 @@
       </c>
       <c r="P31" s="5"/>
     </row>
-    <row r="32" spans="1:17" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:17" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A32" s="21">
         <v>45443</v>
       </c>
@@ -2947,7 +4013,7 @@
       </c>
       <c r="P32" s="5"/>
     </row>
-    <row r="33" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A33" s="21">
         <v>45443</v>
       </c>
@@ -2995,7 +4061,7 @@
       </c>
       <c r="P33" s="5"/>
     </row>
-    <row r="34" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A34" s="21">
         <v>45443</v>
       </c>
@@ -3043,7 +4109,7 @@
       </c>
       <c r="P34" s="5"/>
     </row>
-    <row r="35" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A35" s="21">
         <v>45459</v>
       </c>
@@ -3087,7 +4153,7 @@
       <c r="O35" s="41"/>
       <c r="P35" s="5"/>
     </row>
-    <row r="36" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="21">
         <v>45473</v>
       </c>
@@ -3135,7 +4201,7 @@
       </c>
       <c r="P36" s="5"/>
     </row>
-    <row r="37" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="21">
         <v>45473</v>
       </c>
@@ -3176,7 +4242,7 @@
       </c>
       <c r="P37" s="5"/>
     </row>
-    <row r="38" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A38" s="21">
         <v>45732</v>
       </c>
@@ -3218,7 +4284,7 @@
       <c r="O38" s="5"/>
       <c r="P38" s="5"/>
     </row>
-    <row r="39" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="21">
         <v>45732</v>
       </c>
@@ -3262,7 +4328,7 @@
       </c>
       <c r="P39" s="5"/>
     </row>
-    <row r="40" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A40" s="7">
         <v>45688</v>
       </c>
@@ -3300,7 +4366,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="41" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A41" s="7">
         <v>45688</v>
       </c>
@@ -3338,7 +4404,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A42" s="7">
         <v>45573</v>
       </c>
@@ -3382,7 +4448,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A43" s="7">
         <v>45573</v>
       </c>
@@ -3426,7 +4492,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A44" s="21">
         <v>45399</v>
       </c>
@@ -3468,7 +4534,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A45" s="21">
         <v>45406</v>
       </c>
@@ -3510,7 +4576,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A46" s="21">
         <v>45412</v>
       </c>
@@ -3550,7 +4616,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A47" s="21">
         <v>45412</v>
       </c>
@@ -3590,7 +4656,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A48" s="21">
         <v>45412</v>
       </c>
@@ -3630,7 +4696,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A49" s="21">
         <v>45397</v>
       </c>
@@ -3673,7 +4739,7 @@
       </c>
       <c r="O49" s="5"/>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A50" s="21">
         <v>45427</v>
       </c>
@@ -3718,7 +4784,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A51" s="21">
         <v>45427</v>
       </c>
@@ -3761,7 +4827,7 @@
       </c>
       <c r="O51" s="5"/>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A52" s="21">
         <v>45398</v>
       </c>
@@ -3799,7 +4865,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A53" s="21">
         <v>45398</v>
       </c>
@@ -3837,7 +4903,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A54" s="21">
         <v>45398</v>
       </c>
@@ -3875,7 +4941,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A55" s="21">
         <v>45600</v>
       </c>
@@ -3913,7 +4979,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A56" s="21">
         <v>45630</v>
       </c>
@@ -3951,7 +5017,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="57" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A57" s="21">
         <v>45382</v>
       </c>
@@ -3997,7 +5063,7 @@
       </c>
       <c r="P57" s="5"/>
     </row>
-    <row r="58" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A58" s="21">
         <v>45382</v>
       </c>
@@ -4045,7 +5111,7 @@
       </c>
       <c r="P58" s="5"/>
     </row>
-    <row r="59" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A59" s="21">
         <v>45382</v>
       </c>
@@ -4091,7 +5157,7 @@
       </c>
       <c r="P59" s="5"/>
     </row>
-    <row r="60" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A60" s="21">
         <v>45382</v>
       </c>
@@ -4139,7 +5205,7 @@
       </c>
       <c r="P60" s="5"/>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A61" s="21">
         <v>45430</v>
       </c>
@@ -4179,7 +5245,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A62" s="21">
         <v>45448</v>
       </c>
@@ -4219,7 +5285,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A63" s="21">
         <v>45352</v>
       </c>
@@ -4266,7 +5332,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A64" s="21">
         <v>45356</v>
       </c>
@@ -4313,7 +5379,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="65" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A65" s="21">
         <v>45346</v>
       </c>
@@ -4355,7 +5421,7 @@
       <c r="O65" s="5"/>
       <c r="P65" s="5"/>
     </row>
-    <row r="66" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A66" s="21">
         <v>45350</v>
       </c>
@@ -4403,7 +5469,7 @@
       </c>
       <c r="P66" s="5"/>
     </row>
-    <row r="67" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A67" s="21">
         <v>45350</v>
       </c>
@@ -4451,7 +5517,7 @@
       </c>
       <c r="P67" s="5"/>
     </row>
-    <row r="68" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A68" s="21">
         <v>45382</v>
       </c>
@@ -4498,7 +5564,7 @@
       </c>
       <c r="P68" s="5"/>
     </row>
-    <row r="69" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A69" s="21">
         <v>45371</v>
       </c>
@@ -4540,7 +5606,7 @@
       <c r="O69" s="5"/>
       <c r="P69" s="5"/>
     </row>
-    <row r="70" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A70" s="21">
         <v>45382</v>
       </c>
@@ -4588,7 +5654,7 @@
       </c>
       <c r="P70" s="5"/>
     </row>
-    <row r="71" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A71" s="21">
         <v>45382</v>
       </c>
@@ -4634,7 +5700,7 @@
       </c>
       <c r="P71" s="5"/>
     </row>
-    <row r="72" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A72" s="21">
         <v>45382</v>
       </c>
@@ -4678,7 +5744,7 @@
       <c r="O72" s="5"/>
       <c r="P72" s="5"/>
     </row>
-    <row r="73" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A73" s="21">
         <v>45382</v>
       </c>
@@ -4724,7 +5790,7 @@
       </c>
       <c r="P73" s="5"/>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A74" s="21">
         <v>45382</v>
       </c>
@@ -4771,7 +5837,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A75" s="21">
         <v>45382</v>
       </c>
@@ -4814,7 +5880,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="76" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A76" s="21">
         <v>45382</v>
       </c>
@@ -4862,7 +5928,7 @@
       </c>
       <c r="P76" s="5"/>
     </row>
-    <row r="77" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A77" s="21">
         <v>45398</v>
       </c>
@@ -4906,7 +5972,7 @@
       <c r="O77" s="26"/>
       <c r="P77" s="5"/>
     </row>
-    <row r="78" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A78" s="7">
         <v>45473</v>
       </c>
@@ -4944,7 +6010,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="79" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A79" s="7">
         <v>45473</v>
       </c>
@@ -4982,7 +6048,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A80" s="21">
         <v>45351</v>
       </c>
@@ -5024,7 +6090,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A81" s="21">
         <v>45351</v>
       </c>
@@ -5066,7 +6132,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A82" s="21">
         <v>45351</v>
       </c>
@@ -5108,7 +6174,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A83" s="21">
         <v>45370</v>
       </c>
@@ -5150,7 +6216,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A84" s="21">
         <v>45342</v>
       </c>
@@ -5192,7 +6258,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A85" s="21">
         <v>45374</v>
       </c>
@@ -5234,7 +6300,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="86" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A86" s="21">
         <v>45350</v>
       </c>
@@ -5278,7 +6344,7 @@
       <c r="O86" s="5"/>
       <c r="P86" s="5"/>
     </row>
-    <row r="87" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A87" s="21">
         <v>45350</v>
       </c>
@@ -5322,7 +6388,7 @@
       <c r="O87" s="5"/>
       <c r="P87" s="5"/>
     </row>
-    <row r="88" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:16" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A88" s="15">
         <v>45353</v>
       </c>
@@ -5368,7 +6434,7 @@
       </c>
       <c r="P88" s="5"/>
     </row>
-    <row r="89" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A89" s="15">
         <v>45353</v>
       </c>
@@ -5414,7 +6480,7 @@
       </c>
       <c r="P89" s="5"/>
     </row>
-    <row r="90" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A90" s="21">
         <v>45350</v>
       </c>
@@ -5458,7 +6524,7 @@
       <c r="O90" s="5"/>
       <c r="P90" s="5"/>
     </row>
-    <row r="91" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A91" s="21">
         <v>45351</v>
       </c>
@@ -5502,7 +6568,7 @@
       <c r="O91" s="5"/>
       <c r="P91" s="5"/>
     </row>
-    <row r="92" spans="1:16" s="6" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:16" s="6" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A92" s="21">
         <v>45413</v>
       </c>
@@ -5546,7 +6612,7 @@
       </c>
       <c r="P92" s="5"/>
     </row>
-    <row r="93" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:16" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A93" s="47">
         <v>45453</v>
       </c>
@@ -5590,7 +6656,7 @@
       </c>
       <c r="P93" s="5"/>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A94" s="21">
         <v>45408</v>
       </c>
@@ -5632,7 +6698,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A95" s="21">
         <v>45417</v>
       </c>
@@ -5677,5 +6743,507 @@
   </sheetData>
   <autoFilter ref="A1:O1" xr:uid="{4FD43689-4205-4B1F-A2C0-F6B0035B0816}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K000000 This document is classified as EOLO - C2 General</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5C76FB9-F6E4-D547-94B0-0C5703D7E041}">
+  <dimension ref="B1:F28"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" style="54"/>
+    <col min="2" max="2" width="3.5" style="54" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" style="54" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="59.1640625" style="57" customWidth="1"/>
+    <col min="5" max="5" width="46.1640625" style="57" customWidth="1"/>
+    <col min="6" max="6" width="73.83203125" style="54" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="10.83203125" style="54"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:6" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B1" s="51" t="s">
+        <v>294</v>
+      </c>
+      <c r="C1" s="51" t="s">
+        <v>295</v>
+      </c>
+      <c r="D1" s="52" t="s">
+        <v>296</v>
+      </c>
+      <c r="E1" s="52" t="s">
+        <v>297</v>
+      </c>
+      <c r="F1" s="53" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="2" spans="2:6" ht="35" x14ac:dyDescent="0.25">
+      <c r="B2" s="59">
+        <v>1</v>
+      </c>
+      <c r="C2" s="55" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="60" t="s">
+        <v>299</v>
+      </c>
+      <c r="E2" s="60" t="s">
+        <v>300</v>
+      </c>
+      <c r="F2" s="58" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" ht="35" x14ac:dyDescent="0.25">
+      <c r="B3" s="59">
+        <v>2</v>
+      </c>
+      <c r="C3" s="55" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" s="60" t="s">
+        <v>301</v>
+      </c>
+      <c r="E3" s="60" t="s">
+        <v>302</v>
+      </c>
+      <c r="F3" s="58" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" ht="35" x14ac:dyDescent="0.25">
+      <c r="B4" s="59">
+        <v>3</v>
+      </c>
+      <c r="C4" s="55" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="60" t="s">
+        <v>303</v>
+      </c>
+      <c r="E4" s="60" t="s">
+        <v>304</v>
+      </c>
+      <c r="F4" s="60" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" ht="213.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="59">
+        <v>4</v>
+      </c>
+      <c r="C5" s="55" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="56" t="s">
+        <v>305</v>
+      </c>
+      <c r="E5" s="60" t="s">
+        <v>306</v>
+      </c>
+      <c r="F5" s="61" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" ht="36" x14ac:dyDescent="0.25">
+      <c r="B6" s="59">
+        <v>5</v>
+      </c>
+      <c r="C6" s="55" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="56" t="s">
+        <v>307</v>
+      </c>
+      <c r="E6" s="60" t="s">
+        <v>308</v>
+      </c>
+      <c r="F6" s="58" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" ht="18" x14ac:dyDescent="0.25">
+      <c r="B7" s="59">
+        <v>6</v>
+      </c>
+      <c r="C7" s="55" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" s="60" t="s">
+        <v>309</v>
+      </c>
+      <c r="E7" s="60" t="s">
+        <v>310</v>
+      </c>
+      <c r="F7" s="58" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" ht="18" x14ac:dyDescent="0.25">
+      <c r="B8" s="59">
+        <v>7</v>
+      </c>
+      <c r="C8" s="55" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="60" t="s">
+        <v>311</v>
+      </c>
+      <c r="E8" s="60" t="s">
+        <v>312</v>
+      </c>
+      <c r="F8" s="62" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" ht="18" x14ac:dyDescent="0.25">
+      <c r="B9" s="59">
+        <v>8</v>
+      </c>
+      <c r="C9" s="55" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" s="60" t="s">
+        <v>313</v>
+      </c>
+      <c r="E9" s="60" t="s">
+        <v>314</v>
+      </c>
+      <c r="F9" s="63"/>
+    </row>
+    <row r="10" spans="2:6" ht="35" x14ac:dyDescent="0.25">
+      <c r="B10" s="59">
+        <v>9</v>
+      </c>
+      <c r="C10" s="55" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" s="60" t="s">
+        <v>315</v>
+      </c>
+      <c r="E10" s="60" t="s">
+        <v>316</v>
+      </c>
+      <c r="F10" s="58" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" ht="35" x14ac:dyDescent="0.25">
+      <c r="B11" s="59">
+        <v>10</v>
+      </c>
+      <c r="C11" s="55" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="60" t="s">
+        <v>317</v>
+      </c>
+      <c r="E11" s="60" t="s">
+        <v>318</v>
+      </c>
+      <c r="F11" s="58" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" ht="18" x14ac:dyDescent="0.25">
+      <c r="B12" s="59">
+        <v>11</v>
+      </c>
+      <c r="C12" s="55" t="s">
+        <v>319</v>
+      </c>
+      <c r="D12" s="60" t="s">
+        <v>320</v>
+      </c>
+      <c r="E12" s="60" t="s">
+        <v>321</v>
+      </c>
+      <c r="F12" s="58" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" ht="35" x14ac:dyDescent="0.25">
+      <c r="B13" s="59">
+        <v>12</v>
+      </c>
+      <c r="C13" s="55" t="s">
+        <v>319</v>
+      </c>
+      <c r="D13" s="60" t="s">
+        <v>322</v>
+      </c>
+      <c r="E13" s="60" t="s">
+        <v>323</v>
+      </c>
+      <c r="F13" s="58" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" ht="35" x14ac:dyDescent="0.25">
+      <c r="B14" s="59">
+        <v>13</v>
+      </c>
+      <c r="C14" s="55" t="s">
+        <v>319</v>
+      </c>
+      <c r="D14" s="60" t="s">
+        <v>324</v>
+      </c>
+      <c r="E14" s="60" t="s">
+        <v>325</v>
+      </c>
+      <c r="F14" s="58" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" ht="18" x14ac:dyDescent="0.25">
+      <c r="B15" s="59">
+        <v>14</v>
+      </c>
+      <c r="C15" s="55" t="s">
+        <v>6</v>
+      </c>
+      <c r="D15" s="60" t="s">
+        <v>326</v>
+      </c>
+      <c r="E15" s="60" t="s">
+        <v>327</v>
+      </c>
+      <c r="F15" s="58" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" ht="18" x14ac:dyDescent="0.25">
+      <c r="B16" s="59">
+        <v>15</v>
+      </c>
+      <c r="C16" s="55" t="s">
+        <v>7</v>
+      </c>
+      <c r="D16" s="60" t="s">
+        <v>328</v>
+      </c>
+      <c r="E16" s="60" t="s">
+        <v>329</v>
+      </c>
+      <c r="F16" s="58" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" ht="36" x14ac:dyDescent="0.25">
+      <c r="B17" s="59">
+        <v>16</v>
+      </c>
+      <c r="C17" s="55" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" s="60" t="s">
+        <v>330</v>
+      </c>
+      <c r="E17" s="60" t="s">
+        <v>331</v>
+      </c>
+      <c r="F17" s="58" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" ht="18" x14ac:dyDescent="0.25">
+      <c r="B18" s="59">
+        <v>17</v>
+      </c>
+      <c r="C18" s="55" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" s="60" t="s">
+        <v>332</v>
+      </c>
+      <c r="E18" s="60" t="s">
+        <v>333</v>
+      </c>
+      <c r="F18" s="58" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" ht="35" x14ac:dyDescent="0.25">
+      <c r="B19" s="59">
+        <v>18</v>
+      </c>
+      <c r="C19" s="55" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="60" t="s">
+        <v>334</v>
+      </c>
+      <c r="E19" s="60" t="s">
+        <v>335</v>
+      </c>
+      <c r="F19" s="58" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" ht="18" x14ac:dyDescent="0.25">
+      <c r="B20" s="59">
+        <v>19</v>
+      </c>
+      <c r="C20" s="55" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="56" t="s">
+        <v>336</v>
+      </c>
+      <c r="E20" s="60" t="s">
+        <v>314</v>
+      </c>
+      <c r="F20" s="58" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" ht="35" x14ac:dyDescent="0.25">
+      <c r="B21" s="59">
+        <v>20</v>
+      </c>
+      <c r="C21" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="60" t="s">
+        <v>337</v>
+      </c>
+      <c r="E21" s="60" t="s">
+        <v>338</v>
+      </c>
+      <c r="F21" s="58" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" ht="35" x14ac:dyDescent="0.25">
+      <c r="B22" s="59">
+        <v>21</v>
+      </c>
+      <c r="C22" s="55" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" s="60" t="s">
+        <v>339</v>
+      </c>
+      <c r="E22" s="60" t="s">
+        <v>340</v>
+      </c>
+      <c r="F22" s="58" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" ht="54" x14ac:dyDescent="0.25">
+      <c r="B23" s="59">
+        <v>22</v>
+      </c>
+      <c r="C23" s="55" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="60" t="s">
+        <v>341</v>
+      </c>
+      <c r="E23" s="60" t="s">
+        <v>342</v>
+      </c>
+      <c r="F23" s="58" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" ht="54" x14ac:dyDescent="0.25">
+      <c r="B24" s="59">
+        <v>23</v>
+      </c>
+      <c r="C24" s="55" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="56" t="s">
+        <v>343</v>
+      </c>
+      <c r="E24" s="60" t="s">
+        <v>344</v>
+      </c>
+      <c r="F24" s="58" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" ht="35" x14ac:dyDescent="0.25">
+      <c r="B25" s="59">
+        <v>24</v>
+      </c>
+      <c r="C25" s="55" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="60" t="s">
+        <v>345</v>
+      </c>
+      <c r="E25" s="60" t="s">
+        <v>346</v>
+      </c>
+      <c r="F25" s="58" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" ht="18" x14ac:dyDescent="0.25">
+      <c r="B26" s="59">
+        <v>25</v>
+      </c>
+      <c r="C26" s="55" t="s">
+        <v>347</v>
+      </c>
+      <c r="D26" s="60" t="s">
+        <v>348</v>
+      </c>
+      <c r="E26" s="60" t="s">
+        <v>331</v>
+      </c>
+      <c r="F26" s="58" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" ht="35" x14ac:dyDescent="0.25">
+      <c r="B27" s="59">
+        <v>26</v>
+      </c>
+      <c r="C27" s="55" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="60" t="s">
+        <v>349</v>
+      </c>
+      <c r="E27" s="60" t="s">
+        <v>331</v>
+      </c>
+      <c r="F27" s="58" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" ht="35" x14ac:dyDescent="0.25">
+      <c r="B28" s="59">
+        <v>27</v>
+      </c>
+      <c r="C28" s="55" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" s="60" t="s">
+        <v>350</v>
+      </c>
+      <c r="E28" s="60" t="s">
+        <v>351</v>
+      </c>
+      <c r="F28" s="58" t="s">
+        <v>375</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="F8:F9"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K000000 This document is classified as EOLO - C2 General</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>